<commit_message>
data(topics): merge T0 into T5 instead of T8
</commit_message>
<xml_diff>
--- a/data/topics/topics_to_name.xlsx
+++ b/data/topics/topics_to_name.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Code\ewallet-review-analysis\data\topics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29E2C6BC-8A49-49C4-B824-43BD4FDB80D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E92B53C-AA95-4D92-A6E6-4F8315B35659}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1507,7 +1507,7 @@
       </c>
       <c r="M3" s="5"/>
       <c r="N3" s="5">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="O3" s="5"/>
     </row>

</xml_diff>